<commit_message>
Synchronize final supplementary tables and source sheets
</commit_message>
<xml_diff>
--- a/Table_S1.xlsx
+++ b/Table_S1.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1A_motif_effects" sheetId="1" r:id="R90666e9a9f4e4068"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1B_family_summary" sheetId="2" r:id="R99a3a2f6d7a64c67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1A_motif_effects" sheetId="1" r:id="Re8b396ccfa074fc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1B_family_summary" sheetId="2" r:id="R7390f95d3d4a4a47"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -327,7 +327,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="34" style="14" customWidth="1"/>
+    <x:col min="1" max="1" width="32" style="14" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" style="14" customWidth="1"/>
     <x:col min="3" max="3" width="18" style="14" customWidth="1"/>
     <x:col min="4" max="4" width="18" style="14" customWidth="1"/>
@@ -364,10 +364,8 @@
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">lost_after_mutation</x:t>
-        </x:is>
+      <x:c r="A3" s="12" t="str">
+        <x:v>lost_in_design</x:v>
       </x:c>
       <x:c r="B3" s="12" t="n">
         <x:v>60</x:v>
@@ -380,10 +378,8 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">gained_after_mutation</x:t>
-        </x:is>
+      <x:c r="A4" s="12" t="str">
+        <x:v>gained_in_design</x:v>
       </x:c>
       <x:c r="B4" s="12" t="n">
         <x:v>50</x:v>
@@ -396,10 +392,8 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">weakened_after_mutation</x:t>
-        </x:is>
+      <x:c r="A5" s="12" t="str">
+        <x:v>weakened_in_design</x:v>
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:v>2</x:v>
@@ -412,10 +406,8 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">strengthened_after_mutation</x:t>
-        </x:is>
+      <x:c r="A6" s="12" t="str">
+        <x:v>strengthened_in_design</x:v>
       </x:c>
       <x:c r="B6" s="12" t="n">
         <x:v>3</x:v>
@@ -489,7 +481,7 @@
   <x:cols>
     <x:col min="1" max="1" width="34" style="14" customWidth="1"/>
     <x:col min="2" max="2" width="18" style="14" customWidth="1"/>
-    <x:col min="3" max="3" width="18" style="14" customWidth="1"/>
+    <x:col min="3" max="3" width="26" style="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="14" customFormat="1" ht="36" customHeight="1">
@@ -510,10 +502,8 @@
           <x:t xml:space="preserve">Native motif-position hits</x:t>
         </x:is>
       </x:c>
-      <x:c r="C2" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Mutated motif-position hits</x:t>
-        </x:is>
+      <x:c r="C2" s="10" t="str">
+        <x:v>Designed HSE-disrupted motif-position hits</x:v>
       </x:c>
     </x:row>
     <x:row r="3">

</xml_diff>